<commit_message>
Add 4 GIMP-style FX, editable Step in Parameter Ranges editor, and several bug fixes
- New common FX: Posterize, Solarize, Pixelate/Mosaic, Edge Detect (Sobel)
- Parameter Ranges editor: Step (slider increment) now editable alongside
  Min/Max, with live in-app refresh on save (no reload needed)
- Fix search filter in Parameter Ranges editor collapsing rows to 3 lines
  after filtering (explicit display:'grid'/'none' instead of '')
- Fix ParticlesGenerator (Magic Sparks) converging onto fixed paths instead
  of moving independently (per-particle noise offsets + time drift)
- Fix LFO Automation min/max/timePct inputs ignoring an explicit 0 value
  (falsy-zero bug in the change handlers)
- Layers preset import dropdown: replace flat <select> with a collapsible
  accordion picker grouped by generator type, so ~260 presets no longer
  need to be scanned as one long list
- New presets: Lissajous Orbit06, Magic Sparks08, Neon Horizon07
</commit_message>
<xml_diff>
--- a/Excels/ParameterRanges.xlsx
+++ b/Excels/ParameterRanges.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H243"/>
+  <dimension ref="A1:I243"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -411,7 +411,7 @@
         <v>Label</v>
       </c>
       <c r="D1" t="str">
-        <v>Step</v>
+        <v>Step (Actual)</v>
       </c>
       <c r="E1" t="str">
         <v>Min (Actual)</v>
@@ -420,9 +420,12 @@
         <v>Max (Actual)</v>
       </c>
       <c r="G1" t="str">
+        <v>Step (Reference)</v>
+      </c>
+      <c r="H1" t="str">
         <v>Min (Reference)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Max (Reference)</v>
       </c>
     </row>
@@ -440,15 +443,18 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F2">
         <v>300</v>
       </c>
       <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>10</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>300</v>
       </c>
     </row>
@@ -469,12 +475,15 @@
         <v>0.001</v>
       </c>
       <c r="F3">
-        <v>0.03</v>
+        <v>0.7</v>
       </c>
       <c r="G3">
         <v>0.001</v>
       </c>
       <c r="H3">
+        <v>0.001</v>
+      </c>
+      <c r="I3">
         <v>0.03</v>
       </c>
     </row>
@@ -501,6 +510,9 @@
         <v>0.1</v>
       </c>
       <c r="H4">
+        <v>0.1</v>
+      </c>
+      <c r="I4">
         <v>10</v>
       </c>
     </row>
@@ -515,18 +527,21 @@
         <v>Thickness</v>
       </c>
       <c r="D5">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>20</v>
       </c>
     </row>
@@ -550,9 +565,12 @@
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>1</v>
       </c>
     </row>
@@ -576,9 +594,12 @@
         <v>100</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
         <v>100</v>
       </c>
     </row>
@@ -596,15 +617,18 @@
         <v>1</v>
       </c>
       <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8">
+        <v>250</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
         <v>10</v>
       </c>
-      <c r="F8">
-        <v>700</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
+      <c r="I8">
         <v>350</v>
       </c>
     </row>
@@ -625,12 +649,15 @@
         <v>0.001</v>
       </c>
       <c r="F9">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="G9">
         <v>0.001</v>
       </c>
       <c r="H9">
+        <v>0.001</v>
+      </c>
+      <c r="I9">
         <v>0.02</v>
       </c>
     </row>
@@ -645,18 +672,21 @@
         <v>Speed</v>
       </c>
       <c r="D10">
-        <v>0.1</v>
+        <v>0.001</v>
       </c>
       <c r="E10">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F10">
-        <v>8</v>
+        <v>0.5</v>
       </c>
       <c r="G10">
         <v>0.1</v>
       </c>
       <c r="H10">
+        <v>0.1</v>
+      </c>
+      <c r="I10">
         <v>8</v>
       </c>
     </row>
@@ -671,18 +701,21 @@
         <v>Thickness</v>
       </c>
       <c r="D11">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
         <v>20</v>
       </c>
     </row>
@@ -706,9 +739,12 @@
         <v>1</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
         <v>1</v>
       </c>
     </row>
@@ -735,6 +771,9 @@
         <v>0.1</v>
       </c>
       <c r="H13">
+        <v>0.1</v>
+      </c>
+      <c r="I13">
         <v>2</v>
       </c>
     </row>
@@ -758,9 +797,12 @@
         <v>100</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
         <v>100</v>
       </c>
     </row>
@@ -778,15 +820,18 @@
         <v>5</v>
       </c>
       <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>500</v>
+      </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
+      <c r="H15">
         <v>10</v>
       </c>
-      <c r="F15">
-        <v>300</v>
-      </c>
-      <c r="G15">
-        <v>10</v>
-      </c>
-      <c r="H15">
+      <c r="I15">
         <v>300</v>
       </c>
     </row>
@@ -801,18 +846,21 @@
         <v>Min Size</v>
       </c>
       <c r="D16">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="F16">
         <v>10</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
         <v>10</v>
       </c>
     </row>
@@ -833,12 +881,15 @@
         <v>2</v>
       </c>
       <c r="F17">
-        <v>30</v>
+        <v>500</v>
       </c>
       <c r="G17">
+        <v>0.5</v>
+      </c>
+      <c r="H17">
         <v>2</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>30</v>
       </c>
     </row>
@@ -865,6 +916,9 @@
         <v>0.1</v>
       </c>
       <c r="H18">
+        <v>0.1</v>
+      </c>
+      <c r="I18">
         <v>10</v>
       </c>
     </row>
@@ -888,9 +942,12 @@
         <v>50</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
         <v>50</v>
       </c>
     </row>
@@ -914,9 +971,12 @@
         <v>100</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
         <v>100</v>
       </c>
     </row>
@@ -937,12 +997,15 @@
         <v>1</v>
       </c>
       <c r="F21">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G21">
         <v>1</v>
       </c>
       <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
         <v>20</v>
       </c>
     </row>
@@ -963,12 +1026,15 @@
         <v>1</v>
       </c>
       <c r="F22">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
       <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
         <v>20</v>
       </c>
     </row>
@@ -995,6 +1061,9 @@
         <v>0.1</v>
       </c>
       <c r="H23">
+        <v>0.1</v>
+      </c>
+      <c r="I23">
         <v>5</v>
       </c>
     </row>
@@ -1009,7 +1078,7 @@
         <v>Thickness</v>
       </c>
       <c r="D24">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E24">
         <v>0.5</v>
@@ -1021,6 +1090,9 @@
         <v>0.5</v>
       </c>
       <c r="H24">
+        <v>0.5</v>
+      </c>
+      <c r="I24">
         <v>15</v>
       </c>
     </row>
@@ -1044,9 +1116,12 @@
         <v>400</v>
       </c>
       <c r="G25">
+        <v>5</v>
+      </c>
+      <c r="H25">
         <v>50</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>400</v>
       </c>
     </row>
@@ -1070,9 +1145,12 @@
         <v>3</v>
       </c>
       <c r="G26">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H26">
+        <v>0.5</v>
+      </c>
+      <c r="I26">
         <v>3</v>
       </c>
     </row>
@@ -1096,9 +1174,12 @@
         <v>6.283185307179586</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
         <v>6.283185307179586</v>
       </c>
     </row>
@@ -1122,9 +1203,12 @@
         <v>100</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
         <v>100</v>
       </c>
     </row>
@@ -1148,9 +1232,12 @@
         <v>20000</v>
       </c>
       <c r="G29">
+        <v>100</v>
+      </c>
+      <c r="H29">
         <v>500</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>20000</v>
       </c>
     </row>
@@ -1177,6 +1264,9 @@
         <v>0.5</v>
       </c>
       <c r="H30">
+        <v>0.5</v>
+      </c>
+      <c r="I30">
         <v>10</v>
       </c>
     </row>
@@ -1203,6 +1293,9 @@
         <v>1</v>
       </c>
       <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31">
         <v>20</v>
       </c>
     </row>
@@ -1229,6 +1322,9 @@
         <v>0.1</v>
       </c>
       <c r="H32">
+        <v>0.1</v>
+      </c>
+      <c r="I32">
         <v>3</v>
       </c>
     </row>
@@ -1243,18 +1339,21 @@
         <v>Thickness</v>
       </c>
       <c r="D33">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E33">
         <v>0.5</v>
       </c>
       <c r="F33">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G33">
         <v>0.5</v>
       </c>
       <c r="H33">
+        <v>0.5</v>
+      </c>
+      <c r="I33">
         <v>10</v>
       </c>
     </row>
@@ -1278,9 +1377,12 @@
         <v>500</v>
       </c>
       <c r="G34">
+        <v>10</v>
+      </c>
+      <c r="H34">
         <v>50</v>
       </c>
-      <c r="H34">
+      <c r="I34">
         <v>500</v>
       </c>
     </row>
@@ -1304,9 +1406,12 @@
         <v>100</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35">
         <v>100</v>
       </c>
     </row>
@@ -1330,9 +1435,12 @@
         <v>300</v>
       </c>
       <c r="G36">
+        <v>5</v>
+      </c>
+      <c r="H36">
         <v>10</v>
       </c>
-      <c r="H36">
+      <c r="I36">
         <v>300</v>
       </c>
     </row>
@@ -1356,9 +1464,12 @@
         <v>40</v>
       </c>
       <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="H37">
         <v>2</v>
       </c>
-      <c r="H37">
+      <c r="I37">
         <v>40</v>
       </c>
     </row>
@@ -1382,9 +1493,12 @@
         <v>80</v>
       </c>
       <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
         <v>5</v>
       </c>
-      <c r="H38">
+      <c r="I38">
         <v>80</v>
       </c>
     </row>
@@ -1399,18 +1513,21 @@
         <v>Thickness</v>
       </c>
       <c r="D39">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E39">
         <v>0.5</v>
       </c>
       <c r="F39">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G39">
         <v>0.5</v>
       </c>
       <c r="H39">
+        <v>0.5</v>
+      </c>
+      <c r="I39">
         <v>8</v>
       </c>
     </row>
@@ -1434,9 +1551,12 @@
         <v>45</v>
       </c>
       <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
         <v>-45</v>
       </c>
-      <c r="H40">
+      <c r="I40">
         <v>45</v>
       </c>
     </row>
@@ -1460,9 +1580,12 @@
         <v>100</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
         <v>100</v>
       </c>
     </row>
@@ -1486,9 +1609,12 @@
         <v>10</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
         <v>10</v>
       </c>
     </row>
@@ -1512,9 +1638,12 @@
         <v>35</v>
       </c>
       <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
         <v>5</v>
       </c>
-      <c r="H43">
+      <c r="I43">
         <v>35</v>
       </c>
     </row>
@@ -1538,9 +1667,12 @@
         <v>150</v>
       </c>
       <c r="G44">
+        <v>5</v>
+      </c>
+      <c r="H44">
         <v>10</v>
       </c>
-      <c r="H44">
+      <c r="I44">
         <v>150</v>
       </c>
     </row>
@@ -1555,18 +1687,21 @@
         <v>Thickness</v>
       </c>
       <c r="D45">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E45">
         <v>0.5</v>
       </c>
       <c r="F45">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G45">
         <v>0.5</v>
       </c>
       <c r="H45">
+        <v>0.5</v>
+      </c>
+      <c r="I45">
         <v>10</v>
       </c>
     </row>
@@ -1590,9 +1725,12 @@
         <v>100</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
         <v>100</v>
       </c>
     </row>
@@ -1619,6 +1757,9 @@
         <v>0.5</v>
       </c>
       <c r="H47">
+        <v>0.5</v>
+      </c>
+      <c r="I47">
         <v>10</v>
       </c>
     </row>
@@ -1642,9 +1783,12 @@
         <v>8</v>
       </c>
       <c r="G48">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H48">
+        <v>0.5</v>
+      </c>
+      <c r="I48">
         <v>8</v>
       </c>
     </row>
@@ -1659,18 +1803,21 @@
         <v>Line Weight</v>
       </c>
       <c r="D49">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E49">
         <v>0.5</v>
       </c>
       <c r="F49">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G49">
         <v>0.5</v>
       </c>
       <c r="H49">
+        <v>0.5</v>
+      </c>
+      <c r="I49">
         <v>10</v>
       </c>
     </row>
@@ -1694,9 +1841,12 @@
         <v>400</v>
       </c>
       <c r="G50">
+        <v>5</v>
+      </c>
+      <c r="H50">
         <v>30</v>
       </c>
-      <c r="H50">
+      <c r="I50">
         <v>400</v>
       </c>
     </row>
@@ -1720,9 +1870,12 @@
         <v>100</v>
       </c>
       <c r="G51">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
         <v>100</v>
       </c>
     </row>
@@ -1746,9 +1899,12 @@
         <v>64</v>
       </c>
       <c r="G52">
+        <v>2</v>
+      </c>
+      <c r="H52">
         <v>8</v>
       </c>
-      <c r="H52">
+      <c r="I52">
         <v>64</v>
       </c>
     </row>
@@ -1775,6 +1931,9 @@
         <v>0.1</v>
       </c>
       <c r="H53">
+        <v>0.1</v>
+      </c>
+      <c r="I53">
         <v>5</v>
       </c>
     </row>
@@ -1801,6 +1960,9 @@
         <v>0.5</v>
       </c>
       <c r="H54">
+        <v>0.5</v>
+      </c>
+      <c r="I54">
         <v>10</v>
       </c>
     </row>
@@ -1824,9 +1986,12 @@
         <v>500</v>
       </c>
       <c r="G55">
+        <v>10</v>
+      </c>
+      <c r="H55">
         <v>50</v>
       </c>
-      <c r="H55">
+      <c r="I55">
         <v>500</v>
       </c>
     </row>
@@ -1850,9 +2015,12 @@
         <v>30</v>
       </c>
       <c r="G56">
+        <v>1</v>
+      </c>
+      <c r="H56">
         <v>2</v>
       </c>
-      <c r="H56">
+      <c r="I56">
         <v>30</v>
       </c>
     </row>
@@ -1876,9 +2044,12 @@
         <v>20</v>
       </c>
       <c r="G57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57">
         <v>20</v>
       </c>
     </row>
@@ -1902,9 +2073,12 @@
         <v>100</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
         <v>100</v>
       </c>
     </row>
@@ -1928,9 +2102,12 @@
         <v>400</v>
       </c>
       <c r="G59">
+        <v>5</v>
+      </c>
+      <c r="H59">
         <v>20</v>
       </c>
-      <c r="H59">
+      <c r="I59">
         <v>400</v>
       </c>
     </row>
@@ -1954,9 +2131,12 @@
         <v>5</v>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60">
         <v>5</v>
       </c>
     </row>
@@ -1980,9 +2160,12 @@
         <v>5</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61">
         <v>5</v>
       </c>
     </row>
@@ -2006,9 +2189,12 @@
         <v>5</v>
       </c>
       <c r="G62">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62">
         <v>5</v>
       </c>
     </row>
@@ -2023,18 +2209,21 @@
         <v>Thickness</v>
       </c>
       <c r="D63">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F63">
         <v>15</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H63">
+        <v>1</v>
+      </c>
+      <c r="I63">
         <v>15</v>
       </c>
     </row>
@@ -2058,9 +2247,12 @@
         <v>1</v>
       </c>
       <c r="G64">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
         <v>1</v>
       </c>
     </row>
@@ -2084,9 +2276,12 @@
         <v>100</v>
       </c>
       <c r="G65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
         <v>100</v>
       </c>
     </row>
@@ -2110,9 +2305,12 @@
         <v>80</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
         <v>80</v>
       </c>
     </row>
@@ -2127,18 +2325,21 @@
         <v>Thickness</v>
       </c>
       <c r="D67">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F67">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H67">
+        <v>1</v>
+      </c>
+      <c r="I67">
         <v>10</v>
       </c>
     </row>
@@ -2162,9 +2363,12 @@
         <v>8</v>
       </c>
       <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="H68">
         <v>3</v>
       </c>
-      <c r="H68">
+      <c r="I68">
         <v>8</v>
       </c>
     </row>
@@ -2188,9 +2392,12 @@
         <v>200</v>
       </c>
       <c r="G69">
+        <v>5</v>
+      </c>
+      <c r="H69">
         <v>10</v>
       </c>
-      <c r="H69">
+      <c r="I69">
         <v>200</v>
       </c>
     </row>
@@ -2214,9 +2421,12 @@
         <v>0.9</v>
       </c>
       <c r="G70">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
         <v>0.9</v>
       </c>
     </row>
@@ -2240,9 +2450,12 @@
         <v>5</v>
       </c>
       <c r="G71">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H71">
+        <v>0.5</v>
+      </c>
+      <c r="I71">
         <v>5</v>
       </c>
     </row>
@@ -2266,9 +2479,12 @@
         <v>100</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H72">
+        <v>0</v>
+      </c>
+      <c r="I72">
         <v>100</v>
       </c>
     </row>
@@ -2292,9 +2508,12 @@
         <v>50</v>
       </c>
       <c r="G73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H73">
+        <v>0</v>
+      </c>
+      <c r="I73">
         <v>50</v>
       </c>
     </row>
@@ -2318,9 +2537,12 @@
         <v>30</v>
       </c>
       <c r="G74">
+        <v>1</v>
+      </c>
+      <c r="H74">
         <v>8</v>
       </c>
-      <c r="H74">
+      <c r="I74">
         <v>30</v>
       </c>
     </row>
@@ -2344,9 +2566,12 @@
         <v>600</v>
       </c>
       <c r="G75">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="H75">
+        <v>100</v>
+      </c>
+      <c r="I75">
         <v>600</v>
       </c>
     </row>
@@ -2370,9 +2595,12 @@
         <v>2</v>
       </c>
       <c r="G76">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H76">
+        <v>0</v>
+      </c>
+      <c r="I76">
         <v>2</v>
       </c>
     </row>
@@ -2396,9 +2624,12 @@
         <v>0.015</v>
       </c>
       <c r="G77">
+        <v>0.0005</v>
+      </c>
+      <c r="H77">
         <v>0.001</v>
       </c>
-      <c r="H77">
+      <c r="I77">
         <v>0.015</v>
       </c>
     </row>
@@ -2413,18 +2644,21 @@
         <v>Max Thickness</v>
       </c>
       <c r="D78">
+        <v>0.1</v>
+      </c>
+      <c r="E78">
+        <v>0.5</v>
+      </c>
+      <c r="F78">
+        <v>15</v>
+      </c>
+      <c r="G78">
         <v>0.01</v>
       </c>
-      <c r="E78">
+      <c r="H78">
         <v>0.05</v>
       </c>
-      <c r="F78">
-        <v>0.5</v>
-      </c>
-      <c r="G78">
-        <v>0.05</v>
-      </c>
-      <c r="H78">
+      <c r="I78">
         <v>0.5</v>
       </c>
     </row>
@@ -2448,9 +2682,12 @@
         <v>100</v>
       </c>
       <c r="G79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H79">
+        <v>0</v>
+      </c>
+      <c r="I79">
         <v>100</v>
       </c>
     </row>
@@ -2474,9 +2711,12 @@
         <v>200</v>
       </c>
       <c r="G80">
+        <v>5</v>
+      </c>
+      <c r="H80">
         <v>10</v>
       </c>
-      <c r="H80">
+      <c r="I80">
         <v>200</v>
       </c>
     </row>
@@ -2500,9 +2740,12 @@
         <v>15</v>
       </c>
       <c r="G81">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H81">
+        <v>1</v>
+      </c>
+      <c r="I81">
         <v>15</v>
       </c>
     </row>
@@ -2529,6 +2772,9 @@
         <v>0.1</v>
       </c>
       <c r="H82">
+        <v>0.1</v>
+      </c>
+      <c r="I82">
         <v>5</v>
       </c>
     </row>
@@ -2552,9 +2798,12 @@
         <v>500</v>
       </c>
       <c r="G83">
+        <v>10</v>
+      </c>
+      <c r="H83">
         <v>50</v>
       </c>
-      <c r="H83">
+      <c r="I83">
         <v>500</v>
       </c>
     </row>
@@ -2581,6 +2830,9 @@
         <v>1</v>
       </c>
       <c r="H84">
+        <v>1</v>
+      </c>
+      <c r="I84">
         <v>30</v>
       </c>
     </row>
@@ -2604,9 +2856,12 @@
         <v>11</v>
       </c>
       <c r="G85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H85">
+        <v>0</v>
+      </c>
+      <c r="I85">
         <v>11</v>
       </c>
     </row>
@@ -2630,9 +2885,12 @@
         <v>100</v>
       </c>
       <c r="G86">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H86">
+        <v>0</v>
+      </c>
+      <c r="I86">
         <v>100</v>
       </c>
     </row>
@@ -2656,9 +2914,12 @@
         <v>100</v>
       </c>
       <c r="G87">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H87">
+        <v>0</v>
+      </c>
+      <c r="I87">
         <v>100</v>
       </c>
     </row>
@@ -2682,9 +2943,12 @@
         <v>150</v>
       </c>
       <c r="G88">
+        <v>5</v>
+      </c>
+      <c r="H88">
         <v>10</v>
       </c>
-      <c r="H88">
+      <c r="I88">
         <v>150</v>
       </c>
     </row>
@@ -2708,9 +2972,12 @@
         <v>12</v>
       </c>
       <c r="G89">
+        <v>1</v>
+      </c>
+      <c r="H89">
         <v>3</v>
       </c>
-      <c r="H89">
+      <c r="I89">
         <v>12</v>
       </c>
     </row>
@@ -2734,9 +3001,12 @@
         <v>150</v>
       </c>
       <c r="G90">
+        <v>1</v>
+      </c>
+      <c r="H90">
         <v>10</v>
       </c>
-      <c r="H90">
+      <c r="I90">
         <v>150</v>
       </c>
     </row>
@@ -2760,9 +3030,12 @@
         <v>8</v>
       </c>
       <c r="G91">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H91">
+        <v>0.5</v>
+      </c>
+      <c r="I91">
         <v>8</v>
       </c>
     </row>
@@ -2783,12 +3056,15 @@
         <v>0.5</v>
       </c>
       <c r="F92">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G92">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H92">
+        <v>0.5</v>
+      </c>
+      <c r="I92">
         <v>5</v>
       </c>
     </row>
@@ -2812,9 +3088,12 @@
         <v>100</v>
       </c>
       <c r="G93">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H93">
+        <v>0</v>
+      </c>
+      <c r="I93">
         <v>100</v>
       </c>
     </row>
@@ -2838,9 +3117,12 @@
         <v>300</v>
       </c>
       <c r="G94">
+        <v>2</v>
+      </c>
+      <c r="H94">
         <v>50</v>
       </c>
-      <c r="H94">
+      <c r="I94">
         <v>300</v>
       </c>
     </row>
@@ -2864,9 +3146,12 @@
         <v>200</v>
       </c>
       <c r="G95">
+        <v>2</v>
+      </c>
+      <c r="H95">
         <v>10</v>
       </c>
-      <c r="H95">
+      <c r="I95">
         <v>200</v>
       </c>
     </row>
@@ -2890,9 +3175,12 @@
         <v>300</v>
       </c>
       <c r="G96">
+        <v>2</v>
+      </c>
+      <c r="H96">
         <v>10</v>
       </c>
-      <c r="H96">
+      <c r="I96">
         <v>300</v>
       </c>
     </row>
@@ -2919,6 +3207,9 @@
         <v>1</v>
       </c>
       <c r="H97">
+        <v>1</v>
+      </c>
+      <c r="I97">
         <v>30</v>
       </c>
     </row>
@@ -2945,6 +3236,9 @@
         <v>0.1</v>
       </c>
       <c r="H98">
+        <v>0.1</v>
+      </c>
+      <c r="I98">
         <v>4</v>
       </c>
     </row>
@@ -2959,18 +3253,21 @@
         <v>Thickness</v>
       </c>
       <c r="D99">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E99">
         <v>0.5</v>
       </c>
       <c r="F99">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G99">
         <v>0.5</v>
       </c>
       <c r="H99">
+        <v>0.5</v>
+      </c>
+      <c r="I99">
         <v>10</v>
       </c>
     </row>
@@ -2994,9 +3291,12 @@
         <v>100</v>
       </c>
       <c r="G100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H100">
+        <v>0</v>
+      </c>
+      <c r="I100">
         <v>100</v>
       </c>
     </row>
@@ -3023,6 +3323,9 @@
         <v>1</v>
       </c>
       <c r="H101">
+        <v>1</v>
+      </c>
+      <c r="I101">
         <v>5</v>
       </c>
     </row>
@@ -3046,9 +3349,12 @@
         <v>600</v>
       </c>
       <c r="G102">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="H102">
+        <v>100</v>
+      </c>
+      <c r="I102">
         <v>600</v>
       </c>
     </row>
@@ -3072,9 +3378,12 @@
         <v>0.01</v>
       </c>
       <c r="G103">
+        <v>0.0005</v>
+      </c>
+      <c r="H103">
         <v>0.001</v>
       </c>
-      <c r="H103">
+      <c r="I103">
         <v>0.01</v>
       </c>
     </row>
@@ -3101,6 +3410,9 @@
         <v>0.1</v>
       </c>
       <c r="H104">
+        <v>0.1</v>
+      </c>
+      <c r="I104">
         <v>3</v>
       </c>
     </row>
@@ -3124,9 +3436,12 @@
         <v>100</v>
       </c>
       <c r="G105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H105">
+        <v>0</v>
+      </c>
+      <c r="I105">
         <v>100</v>
       </c>
     </row>
@@ -3150,9 +3465,12 @@
         <v>250</v>
       </c>
       <c r="G106">
+        <v>5</v>
+      </c>
+      <c r="H106">
         <v>10</v>
       </c>
-      <c r="H106">
+      <c r="I106">
         <v>250</v>
       </c>
     </row>
@@ -3176,9 +3494,12 @@
         <v>8</v>
       </c>
       <c r="G107">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H107">
+        <v>0.5</v>
+      </c>
+      <c r="I107">
         <v>8</v>
       </c>
     </row>
@@ -3205,6 +3526,9 @@
         <v>0.1</v>
       </c>
       <c r="H108">
+        <v>0.1</v>
+      </c>
+      <c r="I108">
         <v>4</v>
       </c>
     </row>
@@ -3228,9 +3552,12 @@
         <v>80</v>
       </c>
       <c r="G109">
+        <v>1</v>
+      </c>
+      <c r="H109">
         <v>5</v>
       </c>
-      <c r="H109">
+      <c r="I109">
         <v>80</v>
       </c>
     </row>
@@ -3254,9 +3581,12 @@
         <v>11</v>
       </c>
       <c r="G110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H110">
+        <v>0</v>
+      </c>
+      <c r="I110">
         <v>11</v>
       </c>
     </row>
@@ -3280,9 +3610,12 @@
         <v>100</v>
       </c>
       <c r="G111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111">
+        <v>0</v>
+      </c>
+      <c r="I111">
         <v>100</v>
       </c>
     </row>
@@ -3306,9 +3639,12 @@
         <v>100</v>
       </c>
       <c r="G112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H112">
+        <v>0</v>
+      </c>
+      <c r="I112">
         <v>100</v>
       </c>
     </row>
@@ -3332,9 +3668,12 @@
         <v>250</v>
       </c>
       <c r="G113">
+        <v>5</v>
+      </c>
+      <c r="H113">
         <v>10</v>
       </c>
-      <c r="H113">
+      <c r="I113">
         <v>250</v>
       </c>
     </row>
@@ -3358,9 +3697,12 @@
         <v>11</v>
       </c>
       <c r="G114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H114">
+        <v>0</v>
+      </c>
+      <c r="I114">
         <v>11</v>
       </c>
     </row>
@@ -3384,9 +3726,12 @@
         <v>10</v>
       </c>
       <c r="G115">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H115">
+        <v>0.5</v>
+      </c>
+      <c r="I115">
         <v>10</v>
       </c>
     </row>
@@ -3410,9 +3755,12 @@
         <v>0.1</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="H116">
+        <v>0</v>
+      </c>
+      <c r="I116">
         <v>0.1</v>
       </c>
     </row>
@@ -3436,9 +3784,12 @@
         <v>0.1</v>
       </c>
       <c r="G117">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="H117">
+        <v>0</v>
+      </c>
+      <c r="I117">
         <v>0.1</v>
       </c>
     </row>
@@ -3462,9 +3813,12 @@
         <v>0.2</v>
       </c>
       <c r="G118">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="H118">
+        <v>0</v>
+      </c>
+      <c r="I118">
         <v>0.2</v>
       </c>
     </row>
@@ -3488,9 +3842,12 @@
         <v>10</v>
       </c>
       <c r="G119">
+        <v>0.5</v>
+      </c>
+      <c r="H119">
         <v>2</v>
       </c>
-      <c r="H119">
+      <c r="I119">
         <v>10</v>
       </c>
     </row>
@@ -3514,9 +3871,12 @@
         <v>40</v>
       </c>
       <c r="G120">
+        <v>0.5</v>
+      </c>
+      <c r="H120">
         <v>5</v>
       </c>
-      <c r="H120">
+      <c r="I120">
         <v>40</v>
       </c>
     </row>
@@ -3540,9 +3900,12 @@
         <v>100</v>
       </c>
       <c r="G121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H121">
+        <v>0</v>
+      </c>
+      <c r="I121">
         <v>100</v>
       </c>
     </row>
@@ -3566,9 +3929,12 @@
         <v>100</v>
       </c>
       <c r="G122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H122">
+        <v>0</v>
+      </c>
+      <c r="I122">
         <v>100</v>
       </c>
     </row>
@@ -3595,6 +3961,9 @@
         <v>1</v>
       </c>
       <c r="H123">
+        <v>1</v>
+      </c>
+      <c r="I123">
         <v>4</v>
       </c>
     </row>
@@ -3618,9 +3987,12 @@
         <v>4</v>
       </c>
       <c r="G124">
+        <v>0.1</v>
+      </c>
+      <c r="H124">
         <v>0.2</v>
       </c>
-      <c r="H124">
+      <c r="I124">
         <v>4</v>
       </c>
     </row>
@@ -3644,9 +4016,12 @@
         <v>60</v>
       </c>
       <c r="G125">
+        <v>1</v>
+      </c>
+      <c r="H125">
         <v>2</v>
       </c>
-      <c r="H125">
+      <c r="I125">
         <v>60</v>
       </c>
     </row>
@@ -3670,9 +4045,12 @@
         <v>1500</v>
       </c>
       <c r="G126">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="H126">
+        <v>100</v>
+      </c>
+      <c r="I126">
         <v>1500</v>
       </c>
     </row>
@@ -3696,9 +4074,12 @@
         <v>100</v>
       </c>
       <c r="G127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H127">
+        <v>0</v>
+      </c>
+      <c r="I127">
         <v>100</v>
       </c>
     </row>
@@ -3722,9 +4103,12 @@
         <v>100</v>
       </c>
       <c r="G128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H128">
+        <v>0</v>
+      </c>
+      <c r="I128">
         <v>100</v>
       </c>
     </row>
@@ -3748,9 +4132,12 @@
         <v>3</v>
       </c>
       <c r="G129">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H129">
+        <v>0</v>
+      </c>
+      <c r="I129">
         <v>3</v>
       </c>
     </row>
@@ -3774,9 +4161,12 @@
         <v>60</v>
       </c>
       <c r="G130">
+        <v>1</v>
+      </c>
+      <c r="H130">
         <v>5</v>
       </c>
-      <c r="H130">
+      <c r="I130">
         <v>60</v>
       </c>
     </row>
@@ -3800,9 +4190,12 @@
         <v>100</v>
       </c>
       <c r="G131">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
         <v>100</v>
       </c>
     </row>
@@ -3826,9 +4219,12 @@
         <v>100</v>
       </c>
       <c r="G132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
         <v>100</v>
       </c>
     </row>
@@ -3852,9 +4248,12 @@
         <v>20000</v>
       </c>
       <c r="G133">
+        <v>100</v>
+      </c>
+      <c r="H133">
         <v>500</v>
       </c>
-      <c r="H133">
+      <c r="I133">
         <v>20000</v>
       </c>
     </row>
@@ -3878,9 +4277,12 @@
         <v>2</v>
       </c>
       <c r="G134">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
         <v>2</v>
       </c>
     </row>
@@ -3907,6 +4309,9 @@
         <v>1</v>
       </c>
       <c r="H135">
+        <v>1</v>
+      </c>
+      <c r="I135">
         <v>3</v>
       </c>
     </row>
@@ -3930,9 +4335,12 @@
         <v>1500</v>
       </c>
       <c r="G136">
+        <v>10</v>
+      </c>
+      <c r="H136">
         <v>200</v>
       </c>
-      <c r="H136">
+      <c r="I136">
         <v>1500</v>
       </c>
     </row>
@@ -3950,15 +4358,18 @@
         <v>1</v>
       </c>
       <c r="E137">
+        <v>0.5</v>
+      </c>
+      <c r="F137">
+        <v>100</v>
+      </c>
+      <c r="G137">
+        <v>1</v>
+      </c>
+      <c r="H137">
         <v>5</v>
       </c>
-      <c r="F137">
-        <v>100</v>
-      </c>
-      <c r="G137">
-        <v>5</v>
-      </c>
-      <c r="H137">
+      <c r="I137">
         <v>100</v>
       </c>
     </row>
@@ -3982,9 +4393,12 @@
         <v>1</v>
       </c>
       <c r="G138">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H138">
+        <v>0</v>
+      </c>
+      <c r="I138">
         <v>1</v>
       </c>
     </row>
@@ -4008,9 +4422,12 @@
         <v>2</v>
       </c>
       <c r="G139">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H139">
+        <v>0</v>
+      </c>
+      <c r="I139">
         <v>2</v>
       </c>
     </row>
@@ -4034,9 +4451,12 @@
         <v>1</v>
       </c>
       <c r="G140">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H140">
+        <v>0</v>
+      </c>
+      <c r="I140">
         <v>1</v>
       </c>
     </row>
@@ -4060,9 +4480,12 @@
         <v>20</v>
       </c>
       <c r="G141">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H141">
+        <v>0</v>
+      </c>
+      <c r="I141">
         <v>20</v>
       </c>
     </row>
@@ -4086,9 +4509,12 @@
         <v>0.3</v>
       </c>
       <c r="G142">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H142">
+        <v>0</v>
+      </c>
+      <c r="I142">
         <v>0.3</v>
       </c>
     </row>
@@ -4112,9 +4538,12 @@
         <v>0.2</v>
       </c>
       <c r="G143">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H143">
+        <v>0</v>
+      </c>
+      <c r="I143">
         <v>0.2</v>
       </c>
     </row>
@@ -4138,9 +4567,12 @@
         <v>0.3</v>
       </c>
       <c r="G144">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H144">
+        <v>0</v>
+      </c>
+      <c r="I144">
         <v>0.3</v>
       </c>
     </row>
@@ -4164,9 +4596,12 @@
         <v>0.5</v>
       </c>
       <c r="G145">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H145">
+        <v>0</v>
+      </c>
+      <c r="I145">
         <v>0.5</v>
       </c>
     </row>
@@ -4190,9 +4625,12 @@
         <v>100</v>
       </c>
       <c r="G146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H146">
+        <v>0</v>
+      </c>
+      <c r="I146">
         <v>100</v>
       </c>
     </row>
@@ -4216,9 +4654,12 @@
         <v>20000</v>
       </c>
       <c r="G147">
+        <v>100</v>
+      </c>
+      <c r="H147">
         <v>500</v>
       </c>
-      <c r="H147">
+      <c r="I147">
         <v>20000</v>
       </c>
     </row>
@@ -4242,9 +4683,12 @@
         <v>24</v>
       </c>
       <c r="G148">
+        <v>1</v>
+      </c>
+      <c r="H148">
         <v>4</v>
       </c>
-      <c r="H148">
+      <c r="I148">
         <v>24</v>
       </c>
     </row>
@@ -4268,9 +4712,12 @@
         <v>1200</v>
       </c>
       <c r="G149">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="H149">
+        <v>100</v>
+      </c>
+      <c r="I149">
         <v>1200</v>
       </c>
     </row>
@@ -4294,9 +4741,12 @@
         <v>10</v>
       </c>
       <c r="G150">
+        <v>1</v>
+      </c>
+      <c r="H150">
         <v>2</v>
       </c>
-      <c r="H150">
+      <c r="I150">
         <v>10</v>
       </c>
     </row>
@@ -4320,9 +4770,12 @@
         <v>120</v>
       </c>
       <c r="G151">
+        <v>1</v>
+      </c>
+      <c r="H151">
         <v>5</v>
       </c>
-      <c r="H151">
+      <c r="I151">
         <v>120</v>
       </c>
     </row>
@@ -4346,9 +4799,12 @@
         <v>0.6</v>
       </c>
       <c r="G152">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H152">
+        <v>0</v>
+      </c>
+      <c r="I152">
         <v>0.6</v>
       </c>
     </row>
@@ -4372,9 +4828,12 @@
         <v>5</v>
       </c>
       <c r="G153">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H153">
+        <v>0</v>
+      </c>
+      <c r="I153">
         <v>5</v>
       </c>
     </row>
@@ -4398,9 +4857,12 @@
         <v>150</v>
       </c>
       <c r="G154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H154">
+        <v>0</v>
+      </c>
+      <c r="I154">
         <v>150</v>
       </c>
     </row>
@@ -4424,9 +4886,12 @@
         <v>0.5</v>
       </c>
       <c r="G155">
+        <v>0.01</v>
+      </c>
+      <c r="H155">
         <v>0.05</v>
       </c>
-      <c r="H155">
+      <c r="I155">
         <v>0.5</v>
       </c>
     </row>
@@ -4450,9 +4915,12 @@
         <v>0.6</v>
       </c>
       <c r="G156">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H156">
+        <v>0</v>
+      </c>
+      <c r="I156">
         <v>0.6</v>
       </c>
     </row>
@@ -4476,9 +4944,12 @@
         <v>100</v>
       </c>
       <c r="G157">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H157">
+        <v>0</v>
+      </c>
+      <c r="I157">
         <v>100</v>
       </c>
     </row>
@@ -4502,9 +4973,12 @@
         <v>11</v>
       </c>
       <c r="G158">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H158">
+        <v>0</v>
+      </c>
+      <c r="I158">
         <v>11</v>
       </c>
     </row>
@@ -4528,9 +5002,12 @@
         <v>1</v>
       </c>
       <c r="G159">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H159">
+        <v>0</v>
+      </c>
+      <c r="I159">
         <v>1</v>
       </c>
     </row>
@@ -4554,9 +5031,12 @@
         <v>20000</v>
       </c>
       <c r="G160">
+        <v>100</v>
+      </c>
+      <c r="H160">
         <v>500</v>
       </c>
-      <c r="H160">
+      <c r="I160">
         <v>20000</v>
       </c>
     </row>
@@ -4580,9 +5060,12 @@
         <v>360</v>
       </c>
       <c r="G161">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H161">
+        <v>0</v>
+      </c>
+      <c r="I161">
         <v>360</v>
       </c>
     </row>
@@ -4606,9 +5089,12 @@
         <v>48</v>
       </c>
       <c r="G162">
+        <v>1</v>
+      </c>
+      <c r="H162">
         <v>8</v>
       </c>
-      <c r="H162">
+      <c r="I162">
         <v>48</v>
       </c>
     </row>
@@ -4632,9 +5118,12 @@
         <v>1</v>
       </c>
       <c r="G163">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H163">
+        <v>0</v>
+      </c>
+      <c r="I163">
         <v>1</v>
       </c>
     </row>
@@ -4661,6 +5150,9 @@
         <v>1</v>
       </c>
       <c r="H164">
+        <v>1</v>
+      </c>
+      <c r="I164">
         <v>12</v>
       </c>
     </row>
@@ -4684,9 +5176,12 @@
         <v>4</v>
       </c>
       <c r="G165">
+        <v>0.1</v>
+      </c>
+      <c r="H165">
         <v>0.2</v>
       </c>
-      <c r="H165">
+      <c r="I165">
         <v>4</v>
       </c>
     </row>
@@ -4710,9 +5205,12 @@
         <v>30</v>
       </c>
       <c r="G166">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H166">
+        <v>0</v>
+      </c>
+      <c r="I166">
         <v>30</v>
       </c>
     </row>
@@ -4736,9 +5234,12 @@
         <v>1000</v>
       </c>
       <c r="G167">
+        <v>1</v>
+      </c>
+      <c r="H167">
         <v>-1000</v>
       </c>
-      <c r="H167">
+      <c r="I167">
         <v>1000</v>
       </c>
     </row>
@@ -4762,9 +5263,12 @@
         <v>1000</v>
       </c>
       <c r="G168">
+        <v>1</v>
+      </c>
+      <c r="H168">
         <v>-1000</v>
       </c>
-      <c r="H168">
+      <c r="I168">
         <v>1000</v>
       </c>
     </row>
@@ -4788,9 +5292,12 @@
         <v>90</v>
       </c>
       <c r="G169">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H169">
+        <v>0</v>
+      </c>
+      <c r="I169">
         <v>90</v>
       </c>
     </row>
@@ -4814,9 +5321,12 @@
         <v>100</v>
       </c>
       <c r="G170">
+        <v>1</v>
+      </c>
+      <c r="H170">
         <v>20</v>
       </c>
-      <c r="H170">
+      <c r="I170">
         <v>100</v>
       </c>
     </row>
@@ -4840,9 +5350,12 @@
         <v>1</v>
       </c>
       <c r="G171">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H171">
+        <v>0</v>
+      </c>
+      <c r="I171">
         <v>1</v>
       </c>
     </row>
@@ -4866,9 +5379,12 @@
         <v>100</v>
       </c>
       <c r="G172">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H172">
+        <v>0</v>
+      </c>
+      <c r="I172">
         <v>100</v>
       </c>
     </row>
@@ -4892,9 +5408,12 @@
         <v>40</v>
       </c>
       <c r="G173">
+        <v>1</v>
+      </c>
+      <c r="H173">
         <v>2</v>
       </c>
-      <c r="H173">
+      <c r="I173">
         <v>40</v>
       </c>
     </row>
@@ -4921,6 +5440,9 @@
         <v>1</v>
       </c>
       <c r="H174">
+        <v>1</v>
+      </c>
+      <c r="I174">
         <v>15</v>
       </c>
     </row>
@@ -4947,6 +5469,9 @@
         <v>5</v>
       </c>
       <c r="H175">
+        <v>5</v>
+      </c>
+      <c r="I175">
         <v>150</v>
       </c>
     </row>
@@ -4970,9 +5495,12 @@
         <v>0.1</v>
       </c>
       <c r="G176">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="H176">
+        <v>0</v>
+      </c>
+      <c r="I176">
         <v>0.1</v>
       </c>
     </row>
@@ -4996,9 +5524,12 @@
         <v>40</v>
       </c>
       <c r="G177">
+        <v>1</v>
+      </c>
+      <c r="H177">
         <v>2</v>
       </c>
-      <c r="H177">
+      <c r="I177">
         <v>40</v>
       </c>
     </row>
@@ -5022,9 +5553,12 @@
         <v>30</v>
       </c>
       <c r="G178">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H178">
+        <v>0</v>
+      </c>
+      <c r="I178">
         <v>30</v>
       </c>
     </row>
@@ -5048,9 +5582,12 @@
         <v>60</v>
       </c>
       <c r="G179">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H179">
+        <v>0</v>
+      </c>
+      <c r="I179">
         <v>60</v>
       </c>
     </row>
@@ -5074,9 +5611,12 @@
         <v>10</v>
       </c>
       <c r="G180">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H180">
+        <v>0</v>
+      </c>
+      <c r="I180">
         <v>10</v>
       </c>
     </row>
@@ -5100,9 +5640,12 @@
         <v>100</v>
       </c>
       <c r="G181">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H181">
+        <v>0</v>
+      </c>
+      <c r="I181">
         <v>100</v>
       </c>
     </row>
@@ -5126,9 +5669,12 @@
         <v>3000</v>
       </c>
       <c r="G182">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H182">
+        <v>100</v>
+      </c>
+      <c r="I182">
         <v>3000</v>
       </c>
     </row>
@@ -5152,9 +5698,12 @@
         <v>6</v>
       </c>
       <c r="G183">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H183">
+        <v>0.5</v>
+      </c>
+      <c r="I183">
         <v>6</v>
       </c>
     </row>
@@ -5178,9 +5727,12 @@
         <v>100</v>
       </c>
       <c r="G184">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H184">
+        <v>0</v>
+      </c>
+      <c r="I184">
         <v>100</v>
       </c>
     </row>
@@ -5204,9 +5756,12 @@
         <v>100</v>
       </c>
       <c r="G185">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H185">
+        <v>0</v>
+      </c>
+      <c r="I185">
         <v>100</v>
       </c>
     </row>
@@ -5230,9 +5785,12 @@
         <v>500</v>
       </c>
       <c r="G186">
+        <v>5</v>
+      </c>
+      <c r="H186">
         <v>30</v>
       </c>
-      <c r="H186">
+      <c r="I186">
         <v>500</v>
       </c>
     </row>
@@ -5256,9 +5814,12 @@
         <v>45</v>
       </c>
       <c r="G187">
+        <v>1</v>
+      </c>
+      <c r="H187">
         <v>2</v>
       </c>
-      <c r="H187">
+      <c r="I187">
         <v>45</v>
       </c>
     </row>
@@ -5282,9 +5843,12 @@
         <v>100</v>
       </c>
       <c r="G188">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H188">
+        <v>0</v>
+      </c>
+      <c r="I188">
         <v>100</v>
       </c>
     </row>
@@ -5308,9 +5872,12 @@
         <v>1</v>
       </c>
       <c r="G189">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H189">
+        <v>0</v>
+      </c>
+      <c r="I189">
         <v>1</v>
       </c>
     </row>
@@ -5334,9 +5901,12 @@
         <v>300</v>
       </c>
       <c r="G190">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H190">
+        <v>0</v>
+      </c>
+      <c r="I190">
         <v>300</v>
       </c>
     </row>
@@ -5360,9 +5930,12 @@
         <v>0.008</v>
       </c>
       <c r="G191">
+        <v>0.0001</v>
+      </c>
+      <c r="H191">
         <v>0.0005</v>
       </c>
-      <c r="H191">
+      <c r="I191">
         <v>0.008</v>
       </c>
     </row>
@@ -5389,6 +5962,9 @@
         <v>0.1</v>
       </c>
       <c r="H192">
+        <v>0.1</v>
+      </c>
+      <c r="I192">
         <v>4</v>
       </c>
     </row>
@@ -5412,9 +5988,12 @@
         <v>100</v>
       </c>
       <c r="G193">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H193">
+        <v>0</v>
+      </c>
+      <c r="I193">
         <v>100</v>
       </c>
     </row>
@@ -5438,9 +6017,12 @@
         <v>3</v>
       </c>
       <c r="G194">
+        <v>0.1</v>
+      </c>
+      <c r="H194">
         <v>0.3</v>
       </c>
-      <c r="H194">
+      <c r="I194">
         <v>3</v>
       </c>
     </row>
@@ -5464,9 +6046,12 @@
         <v>10</v>
       </c>
       <c r="G195">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H195">
+        <v>0</v>
+      </c>
+      <c r="I195">
         <v>10</v>
       </c>
     </row>
@@ -5493,6 +6078,9 @@
         <v>0.1</v>
       </c>
       <c r="H196">
+        <v>0.1</v>
+      </c>
+      <c r="I196">
         <v>6</v>
       </c>
     </row>
@@ -5516,9 +6104,12 @@
         <v>300</v>
       </c>
       <c r="G197">
+        <v>5</v>
+      </c>
+      <c r="H197">
         <v>20</v>
       </c>
-      <c r="H197">
+      <c r="I197">
         <v>300</v>
       </c>
     </row>
@@ -5542,9 +6133,12 @@
         <v>20</v>
       </c>
       <c r="G198">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H198">
+        <v>1</v>
+      </c>
+      <c r="I198">
         <v>20</v>
       </c>
     </row>
@@ -5568,9 +6162,12 @@
         <v>11</v>
       </c>
       <c r="G199">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H199">
+        <v>0</v>
+      </c>
+      <c r="I199">
         <v>11</v>
       </c>
     </row>
@@ -5594,9 +6191,12 @@
         <v>50</v>
       </c>
       <c r="G200">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H200">
+        <v>0</v>
+      </c>
+      <c r="I200">
         <v>50</v>
       </c>
     </row>
@@ -5620,9 +6220,12 @@
         <v>100</v>
       </c>
       <c r="G201">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H201">
+        <v>0</v>
+      </c>
+      <c r="I201">
         <v>100</v>
       </c>
     </row>
@@ -5646,9 +6249,12 @@
         <v>360</v>
       </c>
       <c r="G202">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H202">
+        <v>0</v>
+      </c>
+      <c r="I202">
         <v>360</v>
       </c>
     </row>
@@ -5672,9 +6278,12 @@
         <v>100</v>
       </c>
       <c r="G203">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H203">
+        <v>0</v>
+      </c>
+      <c r="I203">
         <v>100</v>
       </c>
     </row>
@@ -5698,9 +6307,12 @@
         <v>100</v>
       </c>
       <c r="G204">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H204">
+        <v>0</v>
+      </c>
+      <c r="I204">
         <v>100</v>
       </c>
     </row>
@@ -5724,9 +6336,12 @@
         <v>100</v>
       </c>
       <c r="G205">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H205">
+        <v>0</v>
+      </c>
+      <c r="I205">
         <v>100</v>
       </c>
     </row>
@@ -5750,9 +6365,12 @@
         <v>20000</v>
       </c>
       <c r="G206">
+        <v>100</v>
+      </c>
+      <c r="H206">
         <v>500</v>
       </c>
-      <c r="H206">
+      <c r="I206">
         <v>20000</v>
       </c>
     </row>
@@ -5776,9 +6394,12 @@
         <v>20000</v>
       </c>
       <c r="G207">
+        <v>100</v>
+      </c>
+      <c r="H207">
         <v>500</v>
       </c>
-      <c r="H207">
+      <c r="I207">
         <v>20000</v>
       </c>
     </row>
@@ -5802,9 +6423,12 @@
         <v>9999</v>
       </c>
       <c r="G208">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H208">
+        <v>0</v>
+      </c>
+      <c r="I208">
         <v>9999</v>
       </c>
     </row>
@@ -5828,9 +6452,12 @@
         <v>160</v>
       </c>
       <c r="G209">
+        <v>1</v>
+      </c>
+      <c r="H209">
         <v>8</v>
       </c>
-      <c r="H209">
+      <c r="I209">
         <v>160</v>
       </c>
     </row>
@@ -5854,9 +6481,12 @@
         <v>10</v>
       </c>
       <c r="G210">
+        <v>1</v>
+      </c>
+      <c r="H210">
         <v>2</v>
       </c>
-      <c r="H210">
+      <c r="I210">
         <v>10</v>
       </c>
     </row>
@@ -5880,9 +6510,12 @@
         <v>120</v>
       </c>
       <c r="G211">
+        <v>1</v>
+      </c>
+      <c r="H211">
         <v>5</v>
       </c>
-      <c r="H211">
+      <c r="I211">
         <v>120</v>
       </c>
     </row>
@@ -5906,9 +6539,12 @@
         <v>1</v>
       </c>
       <c r="G212">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H212">
+        <v>0</v>
+      </c>
+      <c r="I212">
         <v>1</v>
       </c>
     </row>
@@ -5932,9 +6568,12 @@
         <v>900</v>
       </c>
       <c r="G213">
+        <v>10</v>
+      </c>
+      <c r="H213">
         <v>60</v>
       </c>
-      <c r="H213">
+      <c r="I213">
         <v>900</v>
       </c>
     </row>
@@ -5958,9 +6597,12 @@
         <v>600</v>
       </c>
       <c r="G214">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H214">
+        <v>0</v>
+      </c>
+      <c r="I214">
         <v>600</v>
       </c>
     </row>
@@ -5984,9 +6626,12 @@
         <v>24</v>
       </c>
       <c r="G215">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H215">
+        <v>1</v>
+      </c>
+      <c r="I215">
         <v>24</v>
       </c>
     </row>
@@ -6010,9 +6655,12 @@
         <v>0.6</v>
       </c>
       <c r="G216">
+        <v>0.01</v>
+      </c>
+      <c r="H216">
         <v>0.05</v>
       </c>
-      <c r="H216">
+      <c r="I216">
         <v>0.6</v>
       </c>
     </row>
@@ -6036,9 +6684,12 @@
         <v>50</v>
       </c>
       <c r="G217">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H217">
+        <v>0</v>
+      </c>
+      <c r="I217">
         <v>50</v>
       </c>
     </row>
@@ -6062,9 +6713,12 @@
         <v>2</v>
       </c>
       <c r="G218">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H218">
+        <v>0</v>
+      </c>
+      <c r="I218">
         <v>2</v>
       </c>
     </row>
@@ -6088,9 +6742,12 @@
         <v>1</v>
       </c>
       <c r="G219">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H219">
+        <v>0</v>
+      </c>
+      <c r="I219">
         <v>1</v>
       </c>
     </row>
@@ -6114,9 +6771,12 @@
         <v>3</v>
       </c>
       <c r="G220">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="H220">
+        <v>0.5</v>
+      </c>
+      <c r="I220">
         <v>3</v>
       </c>
     </row>
@@ -6140,9 +6800,12 @@
         <v>2</v>
       </c>
       <c r="G221">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H221">
+        <v>0</v>
+      </c>
+      <c r="I221">
         <v>2</v>
       </c>
     </row>
@@ -6166,9 +6829,12 @@
         <v>90</v>
       </c>
       <c r="G222">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H222">
+        <v>0</v>
+      </c>
+      <c r="I222">
         <v>90</v>
       </c>
     </row>
@@ -6192,9 +6858,12 @@
         <v>40</v>
       </c>
       <c r="G223">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H223">
+        <v>0</v>
+      </c>
+      <c r="I223">
         <v>40</v>
       </c>
     </row>
@@ -6218,9 +6887,12 @@
         <v>100</v>
       </c>
       <c r="G224">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H224">
+        <v>0</v>
+      </c>
+      <c r="I224">
         <v>100</v>
       </c>
     </row>
@@ -6244,9 +6916,12 @@
         <v>20000</v>
       </c>
       <c r="G225">
+        <v>100</v>
+      </c>
+      <c r="H225">
         <v>500</v>
       </c>
-      <c r="H225">
+      <c r="I225">
         <v>20000</v>
       </c>
     </row>
@@ -6270,9 +6945,12 @@
         <v>20000</v>
       </c>
       <c r="G226">
+        <v>100</v>
+      </c>
+      <c r="H226">
         <v>500</v>
       </c>
-      <c r="H226">
+      <c r="I226">
         <v>20000</v>
       </c>
     </row>
@@ -6296,9 +6974,12 @@
         <v>9999</v>
       </c>
       <c r="G227">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H227">
+        <v>0</v>
+      </c>
+      <c r="I227">
         <v>9999</v>
       </c>
     </row>
@@ -6322,9 +7003,12 @@
         <v>160</v>
       </c>
       <c r="G228">
+        <v>1</v>
+      </c>
+      <c r="H228">
         <v>8</v>
       </c>
-      <c r="H228">
+      <c r="I228">
         <v>160</v>
       </c>
     </row>
@@ -6348,9 +7032,12 @@
         <v>10</v>
       </c>
       <c r="G229">
+        <v>1</v>
+      </c>
+      <c r="H229">
         <v>2</v>
       </c>
-      <c r="H229">
+      <c r="I229">
         <v>10</v>
       </c>
     </row>
@@ -6374,9 +7061,12 @@
         <v>120</v>
       </c>
       <c r="G230">
+        <v>1</v>
+      </c>
+      <c r="H230">
         <v>5</v>
       </c>
-      <c r="H230">
+      <c r="I230">
         <v>120</v>
       </c>
     </row>
@@ -6400,9 +7090,12 @@
         <v>1</v>
       </c>
       <c r="G231">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H231">
+        <v>0</v>
+      </c>
+      <c r="I231">
         <v>1</v>
       </c>
     </row>
@@ -6426,9 +7119,12 @@
         <v>1500</v>
       </c>
       <c r="G232">
+        <v>10</v>
+      </c>
+      <c r="H232">
         <v>60</v>
       </c>
-      <c r="H232">
+      <c r="I232">
         <v>900</v>
       </c>
     </row>
@@ -6452,9 +7148,12 @@
         <v>600</v>
       </c>
       <c r="G233">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H233">
+        <v>0</v>
+      </c>
+      <c r="I233">
         <v>600</v>
       </c>
     </row>
@@ -6478,9 +7177,12 @@
         <v>28</v>
       </c>
       <c r="G234">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H234">
+        <v>1</v>
+      </c>
+      <c r="I234">
         <v>28</v>
       </c>
     </row>
@@ -6504,9 +7206,12 @@
         <v>0.6</v>
       </c>
       <c r="G235">
+        <v>0.01</v>
+      </c>
+      <c r="H235">
         <v>0.05</v>
       </c>
-      <c r="H235">
+      <c r="I235">
         <v>0.6</v>
       </c>
     </row>
@@ -6530,9 +7235,12 @@
         <v>60</v>
       </c>
       <c r="G236">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H236">
+        <v>0</v>
+      </c>
+      <c r="I236">
         <v>60</v>
       </c>
     </row>
@@ -6556,9 +7264,12 @@
         <v>2</v>
       </c>
       <c r="G237">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H237">
+        <v>0</v>
+      </c>
+      <c r="I237">
         <v>2</v>
       </c>
     </row>
@@ -6582,9 +7293,12 @@
         <v>1</v>
       </c>
       <c r="G238">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H238">
+        <v>0</v>
+      </c>
+      <c r="I238">
         <v>1</v>
       </c>
     </row>
@@ -6608,9 +7322,12 @@
         <v>3</v>
       </c>
       <c r="G239">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="H239">
+        <v>0.5</v>
+      </c>
+      <c r="I239">
         <v>3</v>
       </c>
     </row>
@@ -6634,9 +7351,12 @@
         <v>2</v>
       </c>
       <c r="G240">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H240">
+        <v>0</v>
+      </c>
+      <c r="I240">
         <v>2</v>
       </c>
     </row>
@@ -6660,9 +7380,12 @@
         <v>90</v>
       </c>
       <c r="G241">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H241">
+        <v>0</v>
+      </c>
+      <c r="I241">
         <v>90</v>
       </c>
     </row>
@@ -6686,9 +7409,12 @@
         <v>40</v>
       </c>
       <c r="G242">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H242">
+        <v>0</v>
+      </c>
+      <c r="I242">
         <v>40</v>
       </c>
     </row>
@@ -6712,22 +7438,25 @@
         <v>100</v>
       </c>
       <c r="G243">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H243">
+        <v>0</v>
+      </c>
+      <c r="I243">
         <v>100</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H243"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I243"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6737,7 +7466,7 @@
         <v>Label</v>
       </c>
       <c r="C1" t="str">
-        <v>Step</v>
+        <v>Step (Actual)</v>
       </c>
       <c r="D1" t="str">
         <v>Min (Actual)</v>
@@ -6746,9 +7475,12 @@
         <v>Max (Actual)</v>
       </c>
       <c r="F1" t="str">
+        <v>Step (Reference)</v>
+      </c>
+      <c r="G1" t="str">
         <v>Min (Reference)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Max (Reference)</v>
       </c>
     </row>
@@ -6759,6 +7491,9 @@
       <c r="B2" t="str">
         <v>Position X</v>
       </c>
+      <c r="C2">
+        <v>0.01</v>
+      </c>
       <c r="D2">
         <v>-1</v>
       </c>
@@ -6766,9 +7501,12 @@
         <v>1</v>
       </c>
       <c r="F2">
+        <v>0.01</v>
+      </c>
+      <c r="G2">
         <v>-1</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>1</v>
       </c>
     </row>
@@ -6779,6 +7517,9 @@
       <c r="B3" t="str">
         <v>Position Y</v>
       </c>
+      <c r="C3">
+        <v>0.01</v>
+      </c>
       <c r="D3">
         <v>-1</v>
       </c>
@@ -6786,9 +7527,12 @@
         <v>1</v>
       </c>
       <c r="F3">
+        <v>0.01</v>
+      </c>
+      <c r="G3">
         <v>-1</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1</v>
       </c>
     </row>
@@ -6799,6 +7543,9 @@
       <c r="B4" t="str">
         <v>Rotation</v>
       </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
       <c r="D4">
         <v>-360</v>
       </c>
@@ -6806,9 +7553,12 @@
         <v>360</v>
       </c>
       <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
         <v>-360</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>360</v>
       </c>
     </row>
@@ -6819,6 +7569,9 @@
       <c r="B5" t="str">
         <v>Scale</v>
       </c>
+      <c r="C5">
+        <v>0.05</v>
+      </c>
       <c r="D5">
         <v>0.1</v>
       </c>
@@ -6826,9 +7579,12 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G5">
+        <v>0.1</v>
+      </c>
+      <c r="H5">
         <v>5</v>
       </c>
     </row>
@@ -6839,6 +7595,9 @@
       <c r="B6" t="str">
         <v>Strobe Speed</v>
       </c>
+      <c r="C6">
+        <v>0.5</v>
+      </c>
       <c r="D6">
         <v>0</v>
       </c>
@@ -6846,9 +7605,12 @@
         <v>30</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>30</v>
       </c>
     </row>
@@ -6859,6 +7621,9 @@
       <c r="B7" t="str">
         <v>Neon Glow</v>
       </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
       <c r="D7">
         <v>0</v>
       </c>
@@ -6866,9 +7631,12 @@
         <v>100</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>100</v>
       </c>
     </row>
@@ -6879,6 +7647,9 @@
       <c r="B8" t="str">
         <v>Motion Trails</v>
       </c>
+      <c r="C8">
+        <v>0.01</v>
+      </c>
       <c r="D8">
         <v>0</v>
       </c>
@@ -6886,9 +7657,12 @@
         <v>0.95</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>0.95</v>
       </c>
     </row>
@@ -6899,6 +7673,9 @@
       <c r="B9" t="str">
         <v>Trail Spin</v>
       </c>
+      <c r="C9">
+        <v>0.001</v>
+      </c>
       <c r="D9">
         <v>-0.05</v>
       </c>
@@ -6906,9 +7683,12 @@
         <v>0.05</v>
       </c>
       <c r="F9">
+        <v>0.001</v>
+      </c>
+      <c r="G9">
         <v>-0.05</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>0.05</v>
       </c>
     </row>
@@ -6919,6 +7699,9 @@
       <c r="B10" t="str">
         <v>Noise Warp</v>
       </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
       <c r="D10">
         <v>0</v>
       </c>
@@ -6926,9 +7709,12 @@
         <v>40</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
         <v>40</v>
       </c>
     </row>
@@ -6939,6 +7725,9 @@
       <c r="B11" t="str">
         <v>Kaleidoscope</v>
       </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
       <c r="D11">
         <v>0</v>
       </c>
@@ -6946,9 +7735,12 @@
         <v>12</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>12</v>
       </c>
     </row>
@@ -6959,6 +7751,9 @@
       <c r="B12" t="str">
         <v>Mirror Mode</v>
       </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
       <c r="D12">
         <v>0</v>
       </c>
@@ -6966,9 +7761,12 @@
         <v>13</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
         <v>13</v>
       </c>
     </row>
@@ -6979,6 +7777,9 @@
       <c r="B13" t="str">
         <v>Chromatic Aberr</v>
       </c>
+      <c r="C13">
+        <v>0.5</v>
+      </c>
       <c r="D13">
         <v>0</v>
       </c>
@@ -6986,9 +7787,12 @@
         <v>30</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
         <v>30</v>
       </c>
     </row>
@@ -6999,6 +7803,9 @@
       <c r="B14" t="str">
         <v>Hue Rotate</v>
       </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
       <c r="D14">
         <v>-180</v>
       </c>
@@ -7006,9 +7813,12 @@
         <v>180</v>
       </c>
       <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
         <v>-180</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>180</v>
       </c>
     </row>
@@ -7019,6 +7829,9 @@
       <c r="B15" t="str">
         <v>Rotate X</v>
       </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
       <c r="D15">
         <v>-180</v>
       </c>
@@ -7026,9 +7839,12 @@
         <v>180</v>
       </c>
       <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
         <v>-180</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>180</v>
       </c>
     </row>
@@ -7039,6 +7855,9 @@
       <c r="B16" t="str">
         <v>Rotate Y</v>
       </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
       <c r="D16">
         <v>-180</v>
       </c>
@@ -7046,9 +7865,12 @@
         <v>180</v>
       </c>
       <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
         <v>-180</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>180</v>
       </c>
     </row>
@@ -7059,6 +7881,9 @@
       <c r="B17" t="str">
         <v>Rotate Z</v>
       </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
       <c r="D17">
         <v>-180</v>
       </c>
@@ -7066,9 +7891,12 @@
         <v>180</v>
       </c>
       <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
         <v>-180</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>180</v>
       </c>
     </row>
@@ -7079,6 +7907,9 @@
       <c r="B18" t="str">
         <v>Depth (Z)</v>
       </c>
+      <c r="C18">
+        <v>5</v>
+      </c>
       <c r="D18">
         <v>-600</v>
       </c>
@@ -7086,9 +7917,12 @@
         <v>600</v>
       </c>
       <c r="F18">
+        <v>5</v>
+      </c>
+      <c r="G18">
         <v>-600</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>600</v>
       </c>
     </row>
@@ -7099,6 +7933,9 @@
       <c r="B19" t="str">
         <v>Median Blur</v>
       </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
       <c r="D19">
         <v>0</v>
       </c>
@@ -7106,9 +7943,12 @@
         <v>100</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
         <v>100</v>
       </c>
     </row>
@@ -7119,6 +7959,9 @@
       <c r="B20" t="str">
         <v>Emboss</v>
       </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
       <c r="D20">
         <v>0</v>
       </c>
@@ -7126,9 +7969,12 @@
         <v>100</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
         <v>100</v>
       </c>
     </row>
@@ -7139,6 +7985,9 @@
       <c r="B21" t="str">
         <v>Motion Blur</v>
       </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
       <c r="D21">
         <v>0</v>
       </c>
@@ -7146,9 +7995,12 @@
         <v>60</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
         <v>60</v>
       </c>
     </row>
@@ -7159,6 +8011,9 @@
       <c r="B22" t="str">
         <v>Motion Blur Angle</v>
       </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
       <c r="D22">
         <v>0</v>
       </c>
@@ -7166,9 +8021,12 @@
         <v>360</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
         <v>360</v>
       </c>
     </row>
@@ -7179,22 +8037,132 @@
       <c r="B23" t="str">
         <v>Radial Blur</v>
       </c>
+      <c r="C23">
+        <v>0.1</v>
+      </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>edgeDetectIntensity</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Edge Detect</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>100</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>pixelateBlockSize</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Pixelate</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>64</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>posterizeLevels</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Posterize</v>
+      </c>
+      <c r="C26">
+        <v>0.01</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>solarizeThreshold</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Solarize</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>255</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>255</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 more GIMP-style FX: Spherize, Little Planet, Canvas Texture, Paper Tile
- Spherize/Little Planet: per-pixel polar/radial remap FX (fisheye bulge and
  tiny-planet swirl), sharing the existing processAtLowRes downsample scaffold
- Canvas Texture/Paper Tile: cached CanvasPattern overlays painted with
  overlay blending against a 50%-gray base, so only lighter/darker deviations
  from gray affect the frame - reads as a raised/indented physical texture
  without any per-frame recomputation cost
- Wired into FX_PARAM_RANGES, Controls.js fxConfigs, LayerManager's pipeline
  and randomizer exclusion list (grouped with the other manual-only stylize
  FX), Parameter Ranges xlsx/JSON, and paramDescriptions.js (also backfilled
  4 missing descriptions for the previous FX batch: Edge Detect/Pixelate/
  Posterize/Solarize)
</commit_message>
<xml_diff>
--- a/Excels/ParameterRanges.xlsx
+++ b/Excels/ParameterRanges.xlsx
@@ -7456,7 +7456,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8160,9 +8160,113 @@
         <v>255</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>spherizeIntensity</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Spherize</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>100</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>littlePlanetIntensity</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Little Planet</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>100</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>canvasTextureIntensity</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Canvas Texture</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>100</v>
+      </c>
+      <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>paperTileIntensity</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Paper Tile</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>100</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Seamless Tile: scale shift amount with intensity, not just blend width
User-reported: the effect felt like a binary 0/1 toggle instead of a 0-100
dial - the toroidal wrap-shift was hardcoded to exactly half width/height
regardless of intensity, so the dominant visual change (frame jumping into
a hard 4-quadrant swap) was fully present at any intensity > 0. Only the
seam blend band's width scaled with the slider.

Fixed by scaling the shift amount itself with intensity too (0 = no-op,
100 = full half-width shift). Any nonzero shift amount still keeps the
canvas's own outer boundary automatically tileable, so intermediate values
now read as a continuously growing pan-with-wraparound instead of jumping
straight to the full quadrant split. Verified the diff-from-baseline grows
monotonically across intensity 5/15/30/50/70/100 instead of saturating
immediately.
</commit_message>
<xml_diff>
--- a/Excels/ParameterRanges.xlsx
+++ b/Excels/ParameterRanges.xlsx
@@ -1745,13 +1745,13 @@
         <v>Frequency</v>
       </c>
       <c r="D47">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E47">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F47">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G47">
         <v>0.5</v>

</xml_diff>